<commit_message>
DS rigor and dark atp
</commit_message>
<xml_diff>
--- a/Solution_recipes/Pulse_Chase_solutions/Rigor_template.xlsx
+++ b/Solution_recipes/Pulse_Chase_solutions/Rigor_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27726"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Greg Milburn\Documents\solutions\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\utku\GitHub\Protocols\Solution_recipes\Pulse_Chase_solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE75A0E0-CD5A-4985-9834-7CBF3DD54EFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53B997D3-F7AB-4BB8-A04F-E2B34AB2F68D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="30">
   <si>
     <t>Made by</t>
   </si>
@@ -99,9 +99,6 @@
   </si>
   <si>
     <t>Target pH = 6.80</t>
-  </si>
-  <si>
-    <t>Catelog</t>
   </si>
   <si>
     <t>MgCl2 Stock Solution</t>
@@ -199,6 +196,15 @@
   <si>
     <t>Find purity from lot number certificate of analysis (COA) band enter into table to calculate corrected FW</t>
   </si>
+  <si>
+    <t>Catalog</t>
+  </si>
+  <si>
+    <t>Sigma</t>
+  </si>
+  <si>
+    <t>Stock</t>
+  </si>
 </sst>
 </file>
 
@@ -206,8 +212,8 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
-    <numFmt numFmtId="168" formatCode="0.000"/>
-    <numFmt numFmtId="169" formatCode="0.0000"/>
+    <numFmt numFmtId="165" formatCode="0.000"/>
+    <numFmt numFmtId="166" formatCode="0.0000"/>
   </numFmts>
   <fonts count="8" x14ac:knownFonts="1">
     <font>
@@ -265,7 +271,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="17">
+  <borders count="18">
     <border>
       <left/>
       <right/>
@@ -499,11 +505,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -568,28 +585,16 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -613,16 +618,16 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -633,6 +638,27 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -653,9 +679,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -693,7 +719,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -799,7 +825,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -941,7 +967,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -971,13 +997,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="41" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="26"/>
-      <c r="G1" s="43" t="s">
-        <v>26</v>
+      <c r="B1" s="42"/>
+      <c r="C1" s="22"/>
+      <c r="G1" s="39" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -985,9 +1011,9 @@
         <v>0</v>
       </c>
       <c r="B2" s="5"/>
-      <c r="C2" s="27"/>
-      <c r="G2" s="44" t="s">
-        <v>27</v>
+      <c r="C2" s="23"/>
+      <c r="G2" s="40" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -995,7 +1021,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="7"/>
-      <c r="C3" s="28"/>
+      <c r="C3" s="24"/>
     </row>
     <row r="4" spans="1:13" ht="27.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="8" t="s">
@@ -1004,8 +1030,8 @@
       <c r="B4" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="30" t="s">
-        <v>21</v>
+      <c r="C4" s="26" t="s">
+        <v>27</v>
       </c>
       <c r="D4" s="9" t="s">
         <v>4</v>
@@ -1022,17 +1048,17 @@
       <c r="H4" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="I4" s="41" t="s">
+      <c r="I4" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="J4" s="41" t="s">
+      <c r="J4" s="37" t="s">
         <v>8</v>
       </c>
-      <c r="K4" s="42" t="s">
+      <c r="K4" s="38" t="s">
+        <v>23</v>
+      </c>
+      <c r="L4" s="38" t="s">
         <v>24</v>
-      </c>
-      <c r="L4" s="42" t="s">
-        <v>25</v>
       </c>
       <c r="M4" s="10" t="s">
         <v>9</v>
@@ -1042,35 +1068,39 @@
       <c r="A5" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="2"/>
+      <c r="B5" s="2" t="s">
+        <v>28</v>
+      </c>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
       <c r="E5" s="3">
         <v>209.26329999999999</v>
       </c>
-      <c r="F5" s="37"/>
-      <c r="G5" s="3" t="e">
+      <c r="F5" s="33">
+        <v>0.995</v>
+      </c>
+      <c r="G5" s="3">
         <f t="shared" ref="G5:G6" si="0">E5/F5</f>
-        <v>#DIV/0!</v>
+        <v>210.31487437185928</v>
       </c>
       <c r="H5" s="17">
         <v>0.05</v>
       </c>
-      <c r="I5" s="39" t="e">
+      <c r="I5" s="35">
         <f>G5*H5</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J5" s="39" t="e">
+        <v>10.515743718592965</v>
+      </c>
+      <c r="J5" s="35">
         <f t="shared" ref="J5:J10" si="1">I5/2</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K5" s="39" t="e">
+        <v>5.2578718592964826</v>
+      </c>
+      <c r="K5" s="35">
         <f>I5*0.25</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="L5" s="39" t="e">
+        <v>2.6289359296482413</v>
+      </c>
+      <c r="L5" s="35">
         <f>I5*0.1</f>
-        <v>#DIV/0!</v>
+        <v>1.0515743718592965</v>
       </c>
       <c r="M5" s="12"/>
     </row>
@@ -1078,35 +1108,39 @@
       <c r="A6" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="2"/>
+      <c r="B6" s="2" t="s">
+        <v>28</v>
+      </c>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
       <c r="E6" s="3">
         <v>98.15</v>
       </c>
-      <c r="F6" s="37"/>
-      <c r="G6" s="3" t="e">
+      <c r="F6" s="33">
+        <v>0.99</v>
+      </c>
+      <c r="G6" s="3">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>99.141414141414145</v>
       </c>
       <c r="H6" s="17">
         <v>0.12</v>
       </c>
-      <c r="I6" s="39" t="e">
+      <c r="I6" s="35">
         <f>G6*H6</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J6" s="39" t="e">
+        <v>11.896969696969697</v>
+      </c>
+      <c r="J6" s="35">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K6" s="39" t="e">
+        <v>5.9484848484848483</v>
+      </c>
+      <c r="K6" s="35">
         <f t="shared" ref="K6:K10" si="2">I6*0.25</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="L6" s="39" t="e">
+        <v>2.9742424242424241</v>
+      </c>
+      <c r="L6" s="35">
         <f t="shared" ref="L6:L10" si="3">I6*0.1</f>
-        <v>#DIV/0!</v>
+        <v>1.1896969696969697</v>
       </c>
       <c r="M6" s="12"/>
     </row>
@@ -1114,35 +1148,39 @@
       <c r="A7" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="2"/>
+      <c r="B7" s="2" t="s">
+        <v>28</v>
+      </c>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
       <c r="E7" s="2">
         <v>380.35</v>
       </c>
-      <c r="F7" s="37"/>
-      <c r="G7" s="3" t="e">
+      <c r="F7" s="33">
+        <v>0.97899999999999998</v>
+      </c>
+      <c r="G7" s="3">
         <f>E7/F7</f>
-        <v>#DIV/0!</v>
+        <v>388.50868232890707</v>
       </c>
       <c r="H7" s="17">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="I7" s="39" t="e">
+      <c r="I7" s="35">
         <f>G7*H7</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J7" s="39" t="e">
+        <v>1.9425434116445355</v>
+      </c>
+      <c r="J7" s="35">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K7" s="39" t="e">
+        <v>0.97127170582226774</v>
+      </c>
+      <c r="K7" s="35">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="L7" s="39" t="e">
+        <v>0.48563585291113387</v>
+      </c>
+      <c r="L7" s="35">
         <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
+        <v>0.19425434116445356</v>
       </c>
       <c r="M7" s="12"/>
     </row>
@@ -1150,135 +1188,167 @@
       <c r="A8" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="19"/>
-      <c r="C8" s="31"/>
+      <c r="B8" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" s="27"/>
       <c r="D8" s="19"/>
       <c r="E8" s="19">
         <v>154.25299999999999</v>
       </c>
-      <c r="F8" s="37"/>
-      <c r="G8" s="3" t="e">
+      <c r="F8" s="33">
+        <v>0.99</v>
+      </c>
+      <c r="G8" s="3">
         <f>E8/F8</f>
-        <v>#DIV/0!</v>
+        <v>155.8111111111111</v>
       </c>
       <c r="H8" s="20">
         <v>4.0000000000000001E-3</v>
       </c>
-      <c r="I8" s="39" t="e">
+      <c r="I8" s="35">
         <f>G8*H8</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J8" s="39" t="e">
+        <v>0.62324444444444438</v>
+      </c>
+      <c r="J8" s="35">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K8" s="39" t="e">
+        <v>0.31162222222222219</v>
+      </c>
+      <c r="K8" s="35">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="L8" s="39" t="e">
+        <v>0.15581111111111109</v>
+      </c>
+      <c r="L8" s="35">
         <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
+        <v>6.2324444444444439E-2</v>
       </c>
       <c r="M8" s="21"/>
     </row>
     <row r="9" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="B9" s="19"/>
+        <v>22</v>
+      </c>
+      <c r="B9" s="19" t="s">
+        <v>28</v>
+      </c>
       <c r="C9" s="19"/>
       <c r="D9" s="19"/>
       <c r="E9" s="19">
         <v>136.08600000000001</v>
       </c>
-      <c r="F9" s="38"/>
-      <c r="G9" s="3" t="e">
+      <c r="F9" s="34">
+        <v>0.99</v>
+      </c>
+      <c r="G9" s="3">
         <f>E9/F9</f>
-        <v>#DIV/0!</v>
+        <v>137.46060606060607</v>
       </c>
       <c r="H9" s="20">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="I9" s="39" t="e">
+      <c r="I9" s="35">
         <f>G9*H9</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J9" s="39" t="e">
+        <v>0.6873030303030303</v>
+      </c>
+      <c r="J9" s="35">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K9" s="39" t="e">
+        <v>0.34365151515151515</v>
+      </c>
+      <c r="K9" s="35">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="L9" s="39" t="e">
+        <v>0.17182575757575758</v>
+      </c>
+      <c r="L9" s="35">
         <f t="shared" si="3"/>
-        <v>#DIV/0!</v>
+        <v>6.873030303030303E-2</v>
       </c>
       <c r="M9" s="12"/>
     </row>
     <row r="10" spans="1:13" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="32" t="s">
-        <v>22</v>
-      </c>
-      <c r="B10" s="32"/>
-      <c r="C10" s="32"/>
-      <c r="D10" s="33"/>
-      <c r="E10" s="33"/>
-      <c r="F10" s="32"/>
-      <c r="G10" s="34">
+      <c r="A10" s="47" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" s="28" t="s">
+        <v>29</v>
+      </c>
+      <c r="C10" s="28"/>
+      <c r="D10" s="29"/>
+      <c r="E10" s="29"/>
+      <c r="F10" s="28"/>
+      <c r="G10" s="30">
         <v>0.5</v>
       </c>
-      <c r="H10" s="35">
+      <c r="H10" s="31">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="I10" s="40">
+      <c r="I10" s="36">
         <f>((H10*1)/G10)*1000</f>
         <v>10</v>
       </c>
-      <c r="J10" s="40">
+      <c r="J10" s="36">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="K10" s="40">
+      <c r="K10" s="36">
         <f t="shared" si="2"/>
         <v>2.5</v>
       </c>
-      <c r="L10" s="40">
+      <c r="L10" s="36">
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="M10" s="36"/>
+      <c r="M10" s="32"/>
     </row>
-    <row r="11" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="46"/>
+    </row>
     <row r="12" spans="1:13" ht="27.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="24" t="s">
+      <c r="A12" s="43" t="s">
         <v>20</v>
       </c>
-      <c r="B12" s="25"/>
-      <c r="C12" s="29"/>
+      <c r="B12" s="44"/>
+      <c r="C12" s="25"/>
     </row>
     <row r="13" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="13" t="s">
         <v>11</v>
       </c>
       <c r="B13" s="14"/>
-      <c r="C13" s="27"/>
+      <c r="C13" s="23"/>
     </row>
     <row r="14" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="11" t="s">
         <v>12</v>
       </c>
       <c r="B14" s="5"/>
-      <c r="C14" s="27"/>
+      <c r="C14" s="23"/>
+      <c r="H14" s="45"/>
+      <c r="I14" s="45"/>
+      <c r="J14" s="45"/>
+      <c r="K14" s="45"/>
     </row>
     <row r="15" spans="1:13" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A15" s="16" t="s">
         <v>13</v>
       </c>
       <c r="B15" s="15"/>
-      <c r="C15" s="27"/>
+      <c r="C15" s="23"/>
+      <c r="H15" s="45"/>
+      <c r="I15" s="45"/>
+      <c r="J15" s="45"/>
+      <c r="K15" s="45"/>
+    </row>
+    <row r="16" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="H16" s="45"/>
+      <c r="I16" s="45"/>
+      <c r="J16" s="45"/>
+      <c r="K16" s="45"/>
+    </row>
+    <row r="17" spans="8:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="H17" s="45"/>
+      <c r="I17" s="45"/>
+      <c r="J17" s="45"/>
+      <c r="K17" s="45"/>
     </row>
     <row r="38" ht="12.75" x14ac:dyDescent="0.2"/>
     <row r="43" ht="12.75" x14ac:dyDescent="0.2"/>
@@ -1311,11 +1381,35 @@
     <mergeCell ref="A12:B12"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="landscape" r:id="rId1"/>
+  <pageSetup scale="86" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<LabArchives xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:xsd="http://www.w3.org/2001/XMLSchema">
+  <BaseUri>https://mynotebook.labarchives.com</BaseUri>
+  <eid>MTQ1OS45fDY3MzMyMS8xMTIzL0VudHJ5UGFydC8xNTI3NDUzNTcwfDM3MDUuODk5OTk5OTk5OTk5Ng==</eid>
+  <version>1</version>
+  <updated-at>2023-02-07T15:12:35Z</updated-at>
+</LabArchives>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100965EA08FA511AE4C9FFF632E6536ED13" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="abfa450e2c882fa05ec7f6a4b4016779">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5d5a2885-0f9b-4d04-9bc1-f867a2376b8a" xmlns:ns3="6cbc0c5a-d948-46e5-8624-1bad210f77c7" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="53678093842f3275b6926b32e7a9c141" ns2:_="" ns3:_="">
     <xsd:import namespace="5d5a2885-0f9b-4d04-9bc1-f867a2376b8a"/>
@@ -1538,31 +1632,40 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<LabArchives xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:xsd="http://www.w3.org/2001/XMLSchema">
-  <BaseUri>https://mynotebook.labarchives.com</BaseUri>
-  <eid>MTQ1OS45fDY3MzMyMS8xMTIzL0VudHJ5UGFydC8xNTI3NDUzNTcwfDM3MDUuODk5OTk5OTk5OTk5Ng==</eid>
-  <version>1</version>
-  <updated-at>2023-02-07T15:12:35Z</updated-at>
-</LabArchives>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{576E4525-D34E-471F-91EB-AF7A16356FDF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3012E31E-5C99-4C5B-9323-B5D42B3C4F74}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="6cbc0c5a-d948-46e5-8624-1bad210f77c7"/>
+    <ds:schemaRef ds:uri="5d5a2885-0f9b-4d04-9bc1-f867a2376b8a"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{278D5EB4-455C-4B6B-914E-CCAB7C96EAF7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D7A5D5A9-477B-4B97-9F9B-D797D2834A6C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1579,37 +1682,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{278D5EB4-455C-4B6B-914E-CCAB7C96EAF7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3012E31E-5C99-4C5B-9323-B5D42B3C4F74}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="6cbc0c5a-d948-46e5-8624-1bad210f77c7"/>
-    <ds:schemaRef ds:uri="5d5a2885-0f9b-4d04-9bc1-f867a2376b8a"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{576E4525-D34E-471F-91EB-AF7A16356FDF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>